<commit_message>
Fixed Heding in test cases
</commit_message>
<xml_diff>
--- a/Assignment2/GoogleMaps/GoogleMaps_TestCases.xlsx
+++ b/Assignment2/GoogleMaps/GoogleMaps_TestCases.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7500"/>
+    <workbookView windowWidth="20490" windowHeight="7500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="359">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -72,7 +72,7 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>S #</t>
+    <t>S. No.</t>
   </si>
   <si>
     <t>Prerequisites:</t>
@@ -114,7 +114,7 @@
     <t>Actual Results</t>
   </si>
   <si>
-    <t>Pass / Fail / Not executed / Suspended</t>
+    <t xml:space="preserve">Pass / Fail / Not executed </t>
   </si>
   <si>
     <t>Open Google Maps.</t>
@@ -816,6 +816,9 @@
   </si>
   <si>
     <t>Open Google Maps without granting location permission.</t>
+  </si>
+  <si>
+    <t>Pass / Fail / Not executed / Suspended</t>
   </si>
   <si>
     <t>As Expected</t>
@@ -12968,7 +12971,7 @@
       <c r="G19" s="39"/>
       <c r="H19" s="39"/>
       <c r="I19" s="36" t="s">
-        <v>28</v>
+        <v>261</v>
       </c>
       <c r="J19" s="39"/>
       <c r="K19" s="61"/>
@@ -12999,7 +13002,7 @@
       </c>
       <c r="E21" s="21"/>
       <c r="F21" s="30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G21" s="10"/>
       <c r="H21" s="11"/>
@@ -13014,7 +13017,7 @@
         <v>2</v>
       </c>
       <c r="B22" s="44" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="44" t="s">
@@ -13022,7 +13025,7 @@
       </c>
       <c r="E22" s="44"/>
       <c r="F22" s="46" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G22" s="47"/>
       <c r="H22" s="48"/>
@@ -13039,14 +13042,14 @@
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="49" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="5" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G28" s="5"/>
       <c r="H28" s="5"/>
@@ -13189,7 +13192,7 @@
         <v>1</v>
       </c>
       <c r="G36" s="30" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H36" s="10"/>
       <c r="I36" s="10"/>
@@ -13201,7 +13204,7 @@
         <v>2</v>
       </c>
       <c r="B37" s="30" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="11"/>
@@ -13282,7 +13285,7 @@
         <v>20</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C42" s="14"/>
       <c r="D42" s="14"/>
@@ -13329,7 +13332,7 @@
       <c r="G44" s="39"/>
       <c r="H44" s="39"/>
       <c r="I44" s="36" t="s">
-        <v>28</v>
+        <v>261</v>
       </c>
       <c r="J44" s="39"/>
       <c r="K44" s="61"/>
@@ -13360,7 +13363,7 @@
       </c>
       <c r="E46" s="21"/>
       <c r="F46" s="30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G46" s="10"/>
       <c r="H46" s="11"/>
@@ -13379,11 +13382,11 @@
       </c>
       <c r="C47" s="50"/>
       <c r="D47" s="21" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E47" s="21"/>
       <c r="F47" s="30" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G47" s="10"/>
       <c r="H47" s="11"/>
@@ -13398,15 +13401,15 @@
         <v>3</v>
       </c>
       <c r="B48" s="44" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C48" s="45"/>
       <c r="D48" s="44" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E48" s="44"/>
       <c r="F48" s="46" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G48" s="47"/>
       <c r="H48" s="48"/>
@@ -13423,14 +13426,14 @@
       </c>
       <c r="B54" s="2"/>
       <c r="C54" s="51" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E54" s="2"/>
       <c r="F54" s="5" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G54" s="5"/>
       <c r="H54" s="5"/>
@@ -13573,7 +13576,7 @@
         <v>1</v>
       </c>
       <c r="G62" s="30" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H62" s="10"/>
       <c r="I62" s="10"/>
@@ -13585,7 +13588,7 @@
         <v>2</v>
       </c>
       <c r="B63" s="30" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="11"/>
@@ -13666,7 +13669,7 @@
         <v>20</v>
       </c>
       <c r="B68" s="17" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C68" s="14"/>
       <c r="D68" s="14"/>
@@ -13677,7 +13680,7 @@
         <v>22</v>
       </c>
       <c r="I68" s="14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J68" s="14"/>
       <c r="K68" s="55"/>
@@ -13713,7 +13716,7 @@
       <c r="G70" s="39"/>
       <c r="H70" s="39"/>
       <c r="I70" s="36" t="s">
-        <v>28</v>
+        <v>261</v>
       </c>
       <c r="J70" s="39"/>
       <c r="K70" s="61"/>
@@ -13744,7 +13747,7 @@
       </c>
       <c r="E72" s="21"/>
       <c r="F72" s="30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G72" s="10"/>
       <c r="H72" s="11"/>
@@ -13759,15 +13762,15 @@
         <v>2</v>
       </c>
       <c r="B73" s="21" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C73" s="50"/>
       <c r="D73" s="21" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E73" s="21"/>
       <c r="F73" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G73" s="10"/>
       <c r="H73" s="11"/>
@@ -13786,11 +13789,11 @@
       </c>
       <c r="C74" s="45"/>
       <c r="D74" s="44" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E74" s="44"/>
       <c r="F74" s="46" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G74" s="47"/>
       <c r="H74" s="48"/>
@@ -13807,14 +13810,14 @@
       </c>
       <c r="B80" s="2"/>
       <c r="C80" s="49" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E80" s="2"/>
       <c r="F80" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G80" s="5"/>
       <c r="H80" s="5"/>
@@ -13957,7 +13960,7 @@
         <v>1</v>
       </c>
       <c r="G88" s="30" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="H88" s="10"/>
       <c r="I88" s="10"/>
@@ -13969,7 +13972,7 @@
         <v>2</v>
       </c>
       <c r="B89" s="30" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C89" s="10"/>
       <c r="D89" s="11"/>
@@ -14050,7 +14053,7 @@
         <v>20</v>
       </c>
       <c r="B94" s="17" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C94" s="14"/>
       <c r="D94" s="14"/>
@@ -14097,7 +14100,7 @@
       <c r="G96" s="39"/>
       <c r="H96" s="39"/>
       <c r="I96" s="36" t="s">
-        <v>28</v>
+        <v>261</v>
       </c>
       <c r="J96" s="39"/>
       <c r="K96" s="61"/>
@@ -14128,7 +14131,7 @@
       </c>
       <c r="E98" s="21"/>
       <c r="F98" s="30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G98" s="10"/>
       <c r="H98" s="11"/>
@@ -14143,11 +14146,11 @@
         <v>2</v>
       </c>
       <c r="B99" s="21" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C99" s="50"/>
       <c r="D99" s="21" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E99" s="21"/>
       <c r="F99" s="30" t="s">
@@ -14170,11 +14173,11 @@
       </c>
       <c r="C100" s="45"/>
       <c r="D100" s="44" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E100" s="44"/>
       <c r="F100" s="46" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G100" s="47"/>
       <c r="H100" s="48"/>
@@ -14191,14 +14194,14 @@
       </c>
       <c r="B106" s="2"/>
       <c r="C106" s="49" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D106" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E106" s="2"/>
       <c r="F106" s="5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G106" s="5"/>
       <c r="H106" s="5"/>
@@ -14341,7 +14344,7 @@
         <v>1</v>
       </c>
       <c r="G114" s="30" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="H114" s="10"/>
       <c r="I114" s="10"/>
@@ -14353,7 +14356,7 @@
         <v>2</v>
       </c>
       <c r="B115" s="30" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C115" s="10"/>
       <c r="D115" s="11"/>
@@ -14434,7 +14437,7 @@
         <v>20</v>
       </c>
       <c r="B120" s="17" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C120" s="14"/>
       <c r="D120" s="14"/>
@@ -14445,7 +14448,7 @@
         <v>22</v>
       </c>
       <c r="I120" s="14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J120" s="14"/>
       <c r="K120" s="55"/>
@@ -14481,7 +14484,7 @@
       <c r="G122" s="39"/>
       <c r="H122" s="39"/>
       <c r="I122" s="36" t="s">
-        <v>28</v>
+        <v>261</v>
       </c>
       <c r="J122" s="39"/>
       <c r="K122" s="61"/>
@@ -14512,7 +14515,7 @@
       </c>
       <c r="E124" s="21"/>
       <c r="F124" s="30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G124" s="10"/>
       <c r="H124" s="11"/>
@@ -14527,15 +14530,15 @@
         <v>2</v>
       </c>
       <c r="B125" s="21" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C125" s="50"/>
       <c r="D125" s="21" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E125" s="21"/>
       <c r="F125" s="30" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G125" s="10"/>
       <c r="H125" s="11"/>
@@ -14550,15 +14553,15 @@
         <v>3</v>
       </c>
       <c r="B126" s="44" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C126" s="45"/>
       <c r="D126" s="44" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E126" s="44"/>
       <c r="F126" s="46" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G126" s="47"/>
       <c r="H126" s="48"/>
@@ -14575,14 +14578,14 @@
       </c>
       <c r="B132" s="2"/>
       <c r="C132" s="49" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D132" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E132" s="2"/>
       <c r="F132" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G132" s="5"/>
       <c r="H132" s="5"/>
@@ -14725,7 +14728,7 @@
         <v>1</v>
       </c>
       <c r="G140" s="30" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="H140" s="10"/>
       <c r="I140" s="10"/>
@@ -14737,7 +14740,7 @@
         <v>2</v>
       </c>
       <c r="B141" s="30" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C141" s="10"/>
       <c r="D141" s="11"/>
@@ -14818,7 +14821,7 @@
         <v>20</v>
       </c>
       <c r="B146" s="14" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C146" s="14"/>
       <c r="D146" s="14"/>
@@ -14865,7 +14868,7 @@
       <c r="G148" s="39"/>
       <c r="H148" s="39"/>
       <c r="I148" s="36" t="s">
-        <v>28</v>
+        <v>261</v>
       </c>
       <c r="J148" s="39"/>
       <c r="K148" s="61"/>
@@ -14896,7 +14899,7 @@
       </c>
       <c r="E150" s="21"/>
       <c r="F150" s="30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G150" s="10"/>
       <c r="H150" s="11"/>
@@ -14911,15 +14914,15 @@
         <v>2</v>
       </c>
       <c r="B151" s="21" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C151" s="50"/>
       <c r="D151" s="21" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E151" s="21"/>
       <c r="F151" s="30" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G151" s="10"/>
       <c r="H151" s="11"/>
@@ -14934,15 +14937,15 @@
         <v>3</v>
       </c>
       <c r="B152" s="44" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C152" s="45"/>
       <c r="D152" s="44" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E152" s="44"/>
       <c r="F152" s="46" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G152" s="47"/>
       <c r="H152" s="48"/>
@@ -14959,14 +14962,14 @@
       </c>
       <c r="B158" s="2"/>
       <c r="C158" s="49" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D158" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E158" s="2"/>
       <c r="F158" s="5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="G158" s="5"/>
       <c r="H158" s="5"/>
@@ -15109,7 +15112,7 @@
         <v>1</v>
       </c>
       <c r="G166" s="30" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="H166" s="10"/>
       <c r="I166" s="10"/>
@@ -15121,7 +15124,7 @@
         <v>2</v>
       </c>
       <c r="B167" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C167" s="10"/>
       <c r="D167" s="11"/>
@@ -15202,7 +15205,7 @@
         <v>20</v>
       </c>
       <c r="B172" s="17" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C172" s="14"/>
       <c r="D172" s="14"/>
@@ -15249,7 +15252,7 @@
       <c r="G174" s="39"/>
       <c r="H174" s="39"/>
       <c r="I174" s="36" t="s">
-        <v>28</v>
+        <v>261</v>
       </c>
       <c r="J174" s="39"/>
       <c r="K174" s="61"/>
@@ -15280,7 +15283,7 @@
       </c>
       <c r="E176" s="21"/>
       <c r="F176" s="30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G176" s="10"/>
       <c r="H176" s="11"/>
@@ -15295,15 +15298,15 @@
         <v>2</v>
       </c>
       <c r="B177" s="21" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C177" s="50"/>
       <c r="D177" s="21" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E177" s="21"/>
       <c r="F177" s="30" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G177" s="10"/>
       <c r="H177" s="11"/>
@@ -15318,15 +15321,15 @@
         <v>3</v>
       </c>
       <c r="B178" s="44" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C178" s="45"/>
       <c r="D178" s="44" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E178" s="44"/>
       <c r="F178" s="46" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G178" s="47"/>
       <c r="H178" s="48"/>
@@ -15343,14 +15346,14 @@
       </c>
       <c r="B184" s="2"/>
       <c r="C184" s="49" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D184" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E184" s="2"/>
       <c r="F184" s="5" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G184" s="5"/>
       <c r="H184" s="5"/>
@@ -15493,7 +15496,7 @@
         <v>1</v>
       </c>
       <c r="G192" s="30" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="H192" s="10"/>
       <c r="I192" s="10"/>
@@ -15505,7 +15508,7 @@
         <v>2</v>
       </c>
       <c r="B193" s="30" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C193" s="10"/>
       <c r="D193" s="11"/>
@@ -15586,7 +15589,7 @@
         <v>20</v>
       </c>
       <c r="B198" s="14" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C198" s="14"/>
       <c r="D198" s="14"/>
@@ -15633,7 +15636,7 @@
       <c r="G200" s="39"/>
       <c r="H200" s="39"/>
       <c r="I200" s="36" t="s">
-        <v>28</v>
+        <v>261</v>
       </c>
       <c r="J200" s="39"/>
       <c r="K200" s="61"/>
@@ -15664,7 +15667,7 @@
       </c>
       <c r="E202" s="21"/>
       <c r="F202" s="30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G202" s="10"/>
       <c r="H202" s="11"/>
@@ -15679,15 +15682,15 @@
         <v>2</v>
       </c>
       <c r="B203" s="21" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C203" s="50"/>
       <c r="D203" s="21" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E203" s="21"/>
       <c r="F203" s="30" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G203" s="10"/>
       <c r="H203" s="11"/>
@@ -15702,15 +15705,15 @@
         <v>3</v>
       </c>
       <c r="B204" s="44" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C204" s="45"/>
       <c r="D204" s="44" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E204" s="44"/>
       <c r="F204" s="46" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G204" s="47"/>
       <c r="H204" s="48"/>
@@ -15727,14 +15730,14 @@
       </c>
       <c r="B210" s="2"/>
       <c r="C210" s="49" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D210" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E210" s="2"/>
       <c r="F210" s="5" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G210" s="5"/>
       <c r="H210" s="5"/>
@@ -15877,7 +15880,7 @@
         <v>1</v>
       </c>
       <c r="G218" s="30" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H218" s="10"/>
       <c r="I218" s="10"/>
@@ -15889,7 +15892,7 @@
         <v>2</v>
       </c>
       <c r="B219" s="30" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C219" s="10"/>
       <c r="D219" s="11"/>
@@ -15970,7 +15973,7 @@
         <v>20</v>
       </c>
       <c r="B224" s="17" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C224" s="14"/>
       <c r="D224" s="14"/>
@@ -15981,7 +15984,7 @@
         <v>22</v>
       </c>
       <c r="I224" s="14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J224" s="14"/>
       <c r="K224" s="55"/>
@@ -16017,7 +16020,7 @@
       <c r="G226" s="39"/>
       <c r="H226" s="39"/>
       <c r="I226" s="36" t="s">
-        <v>28</v>
+        <v>261</v>
       </c>
       <c r="J226" s="39"/>
       <c r="K226" s="61"/>
@@ -16048,7 +16051,7 @@
       </c>
       <c r="E228" s="21"/>
       <c r="F228" s="30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G228" s="10"/>
       <c r="H228" s="11"/>
@@ -16063,15 +16066,15 @@
         <v>2</v>
       </c>
       <c r="B229" s="21" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C229" s="50"/>
       <c r="D229" s="21" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E229" s="21"/>
       <c r="F229" s="30" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G229" s="10"/>
       <c r="H229" s="11"/>
@@ -16086,15 +16089,15 @@
         <v>3</v>
       </c>
       <c r="B230" s="44" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C230" s="45"/>
       <c r="D230" s="44" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E230" s="44"/>
       <c r="F230" s="46" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G230" s="47"/>
       <c r="H230" s="48"/>
@@ -16111,14 +16114,14 @@
       </c>
       <c r="B236" s="64"/>
       <c r="C236" s="65" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D236" s="66" t="s">
         <v>2</v>
       </c>
       <c r="E236" s="64"/>
       <c r="F236" s="65" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G236" s="65"/>
       <c r="H236" s="65"/>
@@ -16261,7 +16264,7 @@
         <v>1</v>
       </c>
       <c r="G244" s="21" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H244" s="21"/>
       <c r="I244" s="21"/>
@@ -16273,7 +16276,7 @@
         <v>2</v>
       </c>
       <c r="B245" s="21" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C245" s="21"/>
       <c r="D245" s="21"/>
@@ -16292,7 +16295,7 @@
         <v>3</v>
       </c>
       <c r="B246" s="21" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C246" s="21"/>
       <c r="D246" s="21"/>
@@ -16356,7 +16359,7 @@
         <v>20</v>
       </c>
       <c r="B250" s="69" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C250" s="21"/>
       <c r="D250" s="21"/>
@@ -16403,7 +16406,7 @@
       <c r="G252" s="91"/>
       <c r="H252" s="91"/>
       <c r="I252" s="88" t="s">
-        <v>28</v>
+        <v>261</v>
       </c>
       <c r="J252" s="91"/>
       <c r="K252" s="100"/>
@@ -16434,7 +16437,7 @@
       </c>
       <c r="E254" s="21"/>
       <c r="F254" s="21" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G254" s="21"/>
       <c r="H254" s="21"/>
@@ -16449,15 +16452,15 @@
         <v>2</v>
       </c>
       <c r="B255" s="21" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C255" s="50"/>
       <c r="D255" s="21" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E255" s="21"/>
       <c r="F255" s="21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G255" s="21"/>
       <c r="H255" s="21"/>
@@ -16472,15 +16475,15 @@
         <v>3</v>
       </c>
       <c r="B256" s="21" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C256" s="50"/>
       <c r="D256" s="21" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E256" s="21"/>
       <c r="F256" s="21" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G256" s="21"/>
       <c r="H256" s="21"/>

</xml_diff>